<commit_message>
SOTA in all 4 Langs (hell yeah!!!)
</commit_message>
<xml_diff>
--- a/results/metrics.xlsx
+++ b/results/metrics.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ahmadabdullah/Desktop/GHaLIB/results/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1457F9C-BBD8-8844-8E68-0540ECC887E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3BC4F0AD-34A0-9E49-A22B-6301A3F37A73}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="15660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="26">
   <si>
     <t>Sr. No.</t>
   </si>
@@ -1433,8 +1433,12 @@
       <c r="H22" s="6">
         <v>0.7</v>
       </c>
-      <c r="I22" s="6"/>
-      <c r="J22" s="6"/>
+      <c r="I22" s="6">
+        <v>0.7</v>
+      </c>
+      <c r="J22" s="6" t="s">
+        <v>17</v>
+      </c>
       <c r="K22" s="6"/>
       <c r="L22" s="6"/>
       <c r="M22" s="6"/>

</xml_diff>

<commit_message>
add data for conversion
</commit_message>
<xml_diff>
--- a/results/metrics.xlsx
+++ b/results/metrics.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10309"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10315"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ahmadabdullah/Desktop/GHaLIB/results/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3BC4F0AD-34A0-9E49-A22B-6301A3F37A73}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6ACA6404-F944-C840-9E44-094303475B03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="15660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -642,13 +642,13 @@
         <v>6</v>
       </c>
       <c r="G5" s="6">
-        <v>0.73</v>
+        <v>0.77</v>
       </c>
       <c r="H5" s="6">
-        <v>0.53</v>
+        <v>0.66</v>
       </c>
       <c r="I5" s="6">
-        <v>0.53</v>
+        <v>0.66</v>
       </c>
       <c r="J5" s="6" t="s">
         <v>17</v>
@@ -1471,8 +1471,8 @@
       <c r="D23" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="E23" s="8" t="s">
-        <v>9</v>
+      <c r="E23" s="6" t="s">
+        <v>10</v>
       </c>
       <c r="F23" s="6" t="s">
         <v>7</v>

</xml_diff>